<commit_message>
Fix Dataset 3 prompt numbering (v1.0.1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/prompt_derivation.xlsx
+++ b/data/prompt_derivation.xlsx
@@ -5213,7 +5213,7 @@
         <v>3</v>
       </c>
       <c r="B207" s="6" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C207" s="8" t="inlineStr">
         <is>
@@ -5236,7 +5236,7 @@
         <v>3</v>
       </c>
       <c r="B208" s="6" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C208" s="8" t="inlineStr">
         <is>
@@ -5259,7 +5259,7 @@
         <v>3</v>
       </c>
       <c r="B209" s="6" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C209" s="8" t="inlineStr">
         <is>
@@ -5282,7 +5282,7 @@
         <v>3</v>
       </c>
       <c r="B210" s="6" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C210" s="8" t="inlineStr">
         <is>
@@ -5305,7 +5305,7 @@
         <v>3</v>
       </c>
       <c r="B211" s="6" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C211" s="8" t="inlineStr">
         <is>
@@ -5328,7 +5328,7 @@
         <v>3</v>
       </c>
       <c r="B212" s="6" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C212" s="8" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
         <v>3</v>
       </c>
       <c r="B213" s="6" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C213" s="8" t="inlineStr">
         <is>
@@ -5374,7 +5374,7 @@
         <v>3</v>
       </c>
       <c r="B214" s="6" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C214" s="8" t="inlineStr">
         <is>
@@ -5397,7 +5397,7 @@
         <v>3</v>
       </c>
       <c r="B215" s="6" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C215" s="8" t="inlineStr">
         <is>
@@ -5420,7 +5420,7 @@
         <v>3</v>
       </c>
       <c r="B216" s="6" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C216" s="8" t="inlineStr">
         <is>
@@ -5443,7 +5443,7 @@
         <v>3</v>
       </c>
       <c r="B217" s="6" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C217" s="8" t="inlineStr">
         <is>
@@ -5466,7 +5466,7 @@
         <v>3</v>
       </c>
       <c r="B218" s="6" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C218" s="8" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         <v>3</v>
       </c>
       <c r="B219" s="6" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C219" s="8" t="inlineStr">
         <is>
@@ -5512,7 +5512,7 @@
         <v>3</v>
       </c>
       <c r="B220" s="6" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C220" s="8" t="inlineStr">
         <is>
@@ -5535,7 +5535,7 @@
         <v>3</v>
       </c>
       <c r="B221" s="6" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C221" s="8" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
         <v>3</v>
       </c>
       <c r="B222" s="6" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C222" s="8" t="inlineStr">
         <is>
@@ -5581,7 +5581,7 @@
         <v>3</v>
       </c>
       <c r="B223" s="6" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C223" s="8" t="inlineStr">
         <is>
@@ -5604,7 +5604,7 @@
         <v>3</v>
       </c>
       <c r="B224" s="6" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C224" s="8" t="inlineStr">
         <is>
@@ -5627,7 +5627,7 @@
         <v>3</v>
       </c>
       <c r="B225" s="6" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C225" s="8" t="inlineStr">
         <is>
@@ -5650,7 +5650,7 @@
         <v>3</v>
       </c>
       <c r="B226" s="6" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C226" s="8" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
         <v>3</v>
       </c>
       <c r="B227" s="6" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C227" s="8" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         <v>3</v>
       </c>
       <c r="B228" s="6" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C228" s="8" t="inlineStr">
         <is>
@@ -5719,7 +5719,7 @@
         <v>3</v>
       </c>
       <c r="B229" s="6" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C229" s="8" t="inlineStr">
         <is>
@@ -5742,7 +5742,7 @@
         <v>3</v>
       </c>
       <c r="B230" s="6" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C230" s="8" t="inlineStr">
         <is>
@@ -5765,7 +5765,7 @@
         <v>3</v>
       </c>
       <c r="B231" s="6" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C231" s="8" t="inlineStr">
         <is>
@@ -5788,7 +5788,7 @@
         <v>3</v>
       </c>
       <c r="B232" s="6" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C232" s="8" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         <v>3</v>
       </c>
       <c r="B233" s="6" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C233" s="8" t="inlineStr">
         <is>
@@ -5834,7 +5834,7 @@
         <v>3</v>
       </c>
       <c r="B234" s="6" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C234" s="8" t="inlineStr">
         <is>
@@ -5857,7 +5857,7 @@
         <v>3</v>
       </c>
       <c r="B235" s="6" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C235" s="8" t="inlineStr">
         <is>
@@ -5880,7 +5880,7 @@
         <v>3</v>
       </c>
       <c r="B236" s="6" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C236" s="8" t="inlineStr">
         <is>
@@ -5903,7 +5903,7 @@
         <v>3</v>
       </c>
       <c r="B237" s="6" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C237" s="8" t="inlineStr">
         <is>
@@ -5926,7 +5926,7 @@
         <v>3</v>
       </c>
       <c r="B238" s="6" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C238" s="8" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         <v>3</v>
       </c>
       <c r="B239" s="6" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C239" s="8" t="inlineStr">
         <is>
@@ -5972,7 +5972,7 @@
         <v>3</v>
       </c>
       <c r="B240" s="6" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C240" s="8" t="inlineStr">
         <is>
@@ -5995,7 +5995,7 @@
         <v>3</v>
       </c>
       <c r="B241" s="6" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C241" s="8" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         <v>3</v>
       </c>
       <c r="B242" s="6" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C242" s="8" t="inlineStr">
         <is>
@@ -6041,7 +6041,7 @@
         <v>3</v>
       </c>
       <c r="B243" s="6" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C243" s="8" t="inlineStr">
         <is>
@@ -6064,7 +6064,7 @@
         <v>3</v>
       </c>
       <c r="B244" s="6" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C244" s="8" t="inlineStr">
         <is>
@@ -6087,7 +6087,7 @@
         <v>3</v>
       </c>
       <c r="B245" s="6" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C245" s="8" t="inlineStr">
         <is>
@@ -6110,7 +6110,7 @@
         <v>3</v>
       </c>
       <c r="B246" s="6" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C246" s="8" t="inlineStr">
         <is>
@@ -6133,7 +6133,7 @@
         <v>3</v>
       </c>
       <c r="B247" s="6" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C247" s="8" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v>3</v>
       </c>
       <c r="B248" s="6" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C248" s="8" t="inlineStr">
         <is>
@@ -6179,7 +6179,7 @@
         <v>3</v>
       </c>
       <c r="B249" s="6" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C249" s="8" t="inlineStr">
         <is>
@@ -6202,7 +6202,7 @@
         <v>3</v>
       </c>
       <c r="B250" s="6" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C250" s="8" t="inlineStr">
         <is>
@@ -6225,7 +6225,7 @@
         <v>3</v>
       </c>
       <c r="B251" s="6" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C251" s="8" t="inlineStr">
         <is>
@@ -6248,7 +6248,7 @@
         <v>3</v>
       </c>
       <c r="B252" s="6" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C252" s="8" t="inlineStr">
         <is>
@@ -6271,7 +6271,7 @@
         <v>3</v>
       </c>
       <c r="B253" s="6" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C253" s="8" t="inlineStr">
         <is>
@@ -6294,7 +6294,7 @@
         <v>3</v>
       </c>
       <c r="B254" s="6" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C254" s="8" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
         <v>3</v>
       </c>
       <c r="B255" s="6" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C255" s="8" t="inlineStr">
         <is>
@@ -6340,7 +6340,7 @@
         <v>3</v>
       </c>
       <c r="B256" s="6" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C256" s="8" t="inlineStr">
         <is>
@@ -6363,7 +6363,7 @@
         <v>3</v>
       </c>
       <c r="B257" s="6" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C257" s="8" t="inlineStr">
         <is>
@@ -6386,7 +6386,7 @@
         <v>3</v>
       </c>
       <c r="B258" s="6" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C258" s="8" t="inlineStr">
         <is>
@@ -6409,7 +6409,7 @@
         <v>3</v>
       </c>
       <c r="B259" s="6" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C259" s="8" t="inlineStr">
         <is>
@@ -6432,7 +6432,7 @@
         <v>3</v>
       </c>
       <c r="B260" s="6" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C260" s="8" t="inlineStr">
         <is>
@@ -6455,7 +6455,7 @@
         <v>3</v>
       </c>
       <c r="B261" s="9" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C261" s="10" t="inlineStr">
         <is>

</xml_diff>